<commit_message>
making mission profiles work with bat limitations
</commit_message>
<xml_diff>
--- a/reference material/docs/Pathfinder Mission.xlsx
+++ b/reference material/docs/Pathfinder Mission.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johns\Documents (Local_Disk)\Pathfinder-X1\reference material\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{620EF823-9C5C-4868-822F-AD5709D2B86F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E8C0FD-DB51-49FD-9B6F-B261BCE7D43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -250,22 +250,6 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -329,19 +313,35 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="2">
     <tableStyle name="Mission A &amp; B-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
     <tableStyle name="Mission A &amp; B-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1177,11 +1177,11 @@
         <v>28</v>
       </c>
       <c r="B18" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>29</v>
@@ -1261,11 +1261,11 @@
         <v>35</v>
       </c>
       <c r="B20" s="4">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>36</v>
@@ -1388,11 +1388,11 @@
       </c>
       <c r="B23" s="4">
         <f>SUM(B17:B22)</f>
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C23" s="9">
         <f t="shared" si="1"/>
-        <v>1440</v>
+        <v>1080</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>

</xml_diff>